<commit_message>
redundancy: Moorhead clock Mon 13:00 (was 00:00, 250.26 h); totals counted from the first bus, Moorhead 235.76 h
Leaf script, nothing imports it; regress skipped.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy_Moorhead.xlsx
+++ b/docs/redundancy_Moorhead.xlsx
@@ -449,7 +449,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Moorhead: 250.26 h. Miss each ride by one minute and replay the rest.</t>
+          <t>Moorhead: 235.76 h from the first bus. Miss each ride by one minute and replay the rest.</t>
         </is>
       </c>
     </row>
@@ -813,11 +813,11 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d4 Thu 18:55 Greyhound-us: San Bernardino Depot -&gt; Las Vegas Bus Terminal</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
           <t>Oklahoma City</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
+      <c r="E15" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d6 Sat 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+          <t>d6 Sat 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>

</xml_diff>